<commit_message>
feat: revised impossible questions
</commit_message>
<xml_diff>
--- a/lec3/lec3_students_questions.xlsx
+++ b/lec3/lec3_students_questions.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="84">
   <si>
     <t>AI 활용 업무자동화 실습</t>
   </si>
@@ -236,81 +236,6 @@
   </si>
   <si>
     <t xml:space="preserve">  · AI에게 추가로 제공한 정보가 무엇이고, 왜 그걸 제공했는지 설명</t>
-  </si>
-  <si>
-    <t>Q8</t>
-  </si>
-  <si>
-    <t>반복 자동화 — 월간 리포트 템플릿</t>
-  </si>
-  <si>
-    <t>물류팀: "매달 초에 재고 현황 리포트 만드는데 2시간씩 걸려요. 자동화할 수 없을까요?"</t>
-  </si>
-  <si>
-    <t>이 엑셀이 매월 업데이트된다고 가정합니다.</t>
-  </si>
-  <si>
-    <t>다음 달에 새 데이터를 넣어도 동일 품질의 리포트가 나오는</t>
-  </si>
-  <si>
-    <t>"재사용 가능한 프롬프트 템플릿"을 만드세요.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  · 재사용 프롬프트 템플릿 (누가 써도 같은 결과가 나와야 함)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  · 이번 달 샘플 리포트 (템플릿으로 생성한 것)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  · 템플릿 완성까지의 반복 과정 기록</t>
-  </si>
-  <si>
-    <t>Q9</t>
-  </si>
-  <si>
-    <t>AI에게 의사결정 시키기</t>
-  </si>
-  <si>
-    <t>구매팀은 "대량구매로 단가 절감", 재무팀은 "재고 최소화로 현금 확보", 영업팀은 "안전재고 확대로 품절 방지"를 주장합니다.</t>
-  </si>
-  <si>
-    <t>카카오 빈, 대두, 아라비카 원두 3개 품목에 대해</t>
-  </si>
-  <si>
-    <t>AI를 활용하여 각 부서의 주장을 분석하고,</t>
-  </si>
-  <si>
-    <t>본인이 CEO라면 어떤 전략을 택할지 의사결정 보고서를 만드세요.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  · 의사결정 보고서</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  · AI가 만든 부분과 본인이 판단한 부분을 구분하여 표시</t>
-  </si>
-  <si>
-    <t>Q10</t>
-  </si>
-  <si>
-    <t>종합 — 경영진 보고용 대시보드</t>
-  </si>
-  <si>
-    <t>다음 주 월요일 경영회의에서 "수입원자재 현황 및 리스크 브리핑"을 해야 합니다. 발표 10분.</t>
-  </si>
-  <si>
-    <t>AI를 활용하여 경영진 보고용 1페이지 대시보드를 만드세요.</t>
-  </si>
-  <si>
-    <t>1차 시도 → 부족한 점 개선 → 본인의 인사이트 추가하여 최종 완성.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  · 최종 대시보드 (엑셀/PPT/PDF 택1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  · 1차 → 최종까지 프롬프트 변화 과정</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  · "AI가 만든 부분"과 "내가 추가한 부분"을 색으로 구분 표시</t>
   </si>
   <si>
     <t>공통 규칙</t>
@@ -1703,7 +1628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E154"/>
+  <dimension ref="A1:E115"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="4" style="1" customWidth="1"/>
@@ -2649,406 +2574,69 @@
       <c r="E109" s="4"/>
     </row>
     <row r="110" ht="13.55" customHeight="1">
-      <c r="A110" s="7"/>
-      <c r="B110" s="7"/>
-      <c r="C110" s="7"/>
+      <c r="A110" s="3"/>
+      <c r="B110" s="3"/>
+      <c r="C110" s="3"/>
       <c r="D110" s="4"/>
       <c r="E110" s="4"/>
     </row>
-    <row r="111" ht="16.6" customHeight="1">
-      <c r="A111" t="s" s="8">
+    <row r="111" ht="14.6" customHeight="1">
+      <c r="A111" t="s" s="22">
         <v>75</v>
       </c>
-      <c r="B111" t="s" s="9">
+      <c r="B111" s="3"/>
+      <c r="C111" s="3"/>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+    </row>
+    <row r="112" ht="13.55" customHeight="1">
+      <c r="A112" t="s" s="23">
         <v>76</v>
       </c>
-      <c r="C111" t="s" s="21">
-        <v>57</v>
-      </c>
-      <c r="D111" s="11"/>
-      <c r="E111" s="4"/>
-    </row>
-    <row r="112" ht="13.65" customHeight="1">
-      <c r="A112" s="12"/>
-      <c r="B112" t="s" s="13">
+      <c r="B112" t="s" s="24">
         <v>77</v>
       </c>
-      <c r="C112" s="12"/>
+      <c r="C112" s="3"/>
       <c r="D112" s="4"/>
       <c r="E112" s="4"/>
     </row>
     <row r="113" ht="13.55" customHeight="1">
-      <c r="A113" s="3"/>
-      <c r="B113" s="3"/>
+      <c r="A113" t="s" s="23">
+        <v>78</v>
+      </c>
+      <c r="B113" t="s" s="24">
+        <v>79</v>
+      </c>
       <c r="C113" s="3"/>
       <c r="D113" s="4"/>
       <c r="E113" s="4"/>
     </row>
-    <row r="114" ht="13.65" customHeight="1">
-      <c r="A114" s="3"/>
-      <c r="B114" t="s" s="14">
-        <v>78</v>
+    <row r="114" ht="13.55" customHeight="1">
+      <c r="A114" t="s" s="23">
+        <v>80</v>
+      </c>
+      <c r="B114" t="s" s="24">
+        <v>81</v>
       </c>
       <c r="C114" s="3"/>
       <c r="D114" s="4"/>
       <c r="E114" s="4"/>
     </row>
-    <row r="115" ht="13.65" customHeight="1">
-      <c r="A115" s="3"/>
-      <c r="B115" s="15"/>
+    <row r="115" ht="13.55" customHeight="1">
+      <c r="A115" t="s" s="23">
+        <v>82</v>
+      </c>
+      <c r="B115" t="s" s="24">
+        <v>83</v>
+      </c>
       <c r="C115" s="3"/>
       <c r="D115" s="4"/>
       <c r="E115" s="4"/>
     </row>
-    <row r="116" ht="13.65" customHeight="1">
-      <c r="A116" s="3"/>
-      <c r="B116" t="s" s="14">
-        <v>79</v>
-      </c>
-      <c r="C116" s="3"/>
-      <c r="D116" s="4"/>
-      <c r="E116" s="4"/>
-    </row>
-    <row r="117" ht="13.65" customHeight="1">
-      <c r="A117" s="3"/>
-      <c r="B117" t="s" s="14">
-        <v>80</v>
-      </c>
-      <c r="C117" s="3"/>
-      <c r="D117" s="4"/>
-      <c r="E117" s="4"/>
-    </row>
-    <row r="118" ht="13.55" customHeight="1">
-      <c r="A118" s="3"/>
-      <c r="B118" s="7"/>
-      <c r="C118" s="3"/>
-      <c r="D118" s="4"/>
-      <c r="E118" s="4"/>
-    </row>
-    <row r="119" ht="13.65" customHeight="1">
-      <c r="A119" s="16"/>
-      <c r="B119" t="s" s="17">
-        <v>13</v>
-      </c>
-      <c r="C119" s="18"/>
-      <c r="D119" s="4"/>
-      <c r="E119" s="4"/>
-    </row>
-    <row r="120" ht="13.55" customHeight="1">
-      <c r="A120" s="16"/>
-      <c r="B120" t="s" s="19">
-        <v>81</v>
-      </c>
-      <c r="C120" s="18"/>
-      <c r="D120" s="4"/>
-      <c r="E120" s="4"/>
-    </row>
-    <row r="121" ht="13.55" customHeight="1">
-      <c r="A121" s="16"/>
-      <c r="B121" t="s" s="19">
-        <v>82</v>
-      </c>
-      <c r="C121" s="18"/>
-      <c r="D121" s="4"/>
-      <c r="E121" s="4"/>
-    </row>
-    <row r="122" ht="13.55" customHeight="1">
-      <c r="A122" s="16"/>
-      <c r="B122" t="s" s="19">
-        <v>83</v>
-      </c>
-      <c r="C122" s="18"/>
-      <c r="D122" s="4"/>
-      <c r="E122" s="4"/>
-    </row>
-    <row r="123" ht="13.55" customHeight="1">
-      <c r="A123" s="3"/>
-      <c r="B123" s="12"/>
-      <c r="C123" s="3"/>
-      <c r="D123" s="4"/>
-      <c r="E123" s="4"/>
-    </row>
-    <row r="124" ht="13.55" customHeight="1">
-      <c r="A124" s="7"/>
-      <c r="B124" s="7"/>
-      <c r="C124" s="7"/>
-      <c r="D124" s="4"/>
-      <c r="E124" s="4"/>
-    </row>
-    <row r="125" ht="16.6" customHeight="1">
-      <c r="A125" t="s" s="8">
-        <v>84</v>
-      </c>
-      <c r="B125" t="s" s="9">
-        <v>85</v>
-      </c>
-      <c r="C125" t="s" s="21">
-        <v>57</v>
-      </c>
-      <c r="D125" s="11"/>
-      <c r="E125" s="4"/>
-    </row>
-    <row r="126" ht="13.65" customHeight="1">
-      <c r="A126" s="12"/>
-      <c r="B126" t="s" s="13">
-        <v>86</v>
-      </c>
-      <c r="C126" s="12"/>
-      <c r="D126" s="4"/>
-      <c r="E126" s="4"/>
-    </row>
-    <row r="127" ht="13.55" customHeight="1">
-      <c r="A127" s="3"/>
-      <c r="B127" s="3"/>
-      <c r="C127" s="3"/>
-      <c r="D127" s="4"/>
-      <c r="E127" s="4"/>
-    </row>
-    <row r="128" ht="13.65" customHeight="1">
-      <c r="A128" s="3"/>
-      <c r="B128" t="s" s="14">
-        <v>87</v>
-      </c>
-      <c r="C128" s="3"/>
-      <c r="D128" s="4"/>
-      <c r="E128" s="4"/>
-    </row>
-    <row r="129" ht="13.65" customHeight="1">
-      <c r="A129" s="3"/>
-      <c r="B129" t="s" s="14">
-        <v>88</v>
-      </c>
-      <c r="C129" s="3"/>
-      <c r="D129" s="4"/>
-      <c r="E129" s="4"/>
-    </row>
-    <row r="130" ht="13.65" customHeight="1">
-      <c r="A130" s="3"/>
-      <c r="B130" t="s" s="14">
-        <v>89</v>
-      </c>
-      <c r="C130" s="3"/>
-      <c r="D130" s="4"/>
-      <c r="E130" s="4"/>
-    </row>
-    <row r="131" ht="13.55" customHeight="1">
-      <c r="A131" s="3"/>
-      <c r="B131" s="7"/>
-      <c r="C131" s="3"/>
-      <c r="D131" s="4"/>
-      <c r="E131" s="4"/>
-    </row>
-    <row r="132" ht="13.65" customHeight="1">
-      <c r="A132" s="16"/>
-      <c r="B132" t="s" s="17">
-        <v>13</v>
-      </c>
-      <c r="C132" s="18"/>
-      <c r="D132" s="4"/>
-      <c r="E132" s="4"/>
-    </row>
-    <row r="133" ht="13.55" customHeight="1">
-      <c r="A133" s="16"/>
-      <c r="B133" t="s" s="19">
-        <v>90</v>
-      </c>
-      <c r="C133" s="18"/>
-      <c r="D133" s="4"/>
-      <c r="E133" s="4"/>
-    </row>
-    <row r="134" ht="13.55" customHeight="1">
-      <c r="A134" s="16"/>
-      <c r="B134" t="s" s="19">
-        <v>91</v>
-      </c>
-      <c r="C134" s="18"/>
-      <c r="D134" s="4"/>
-      <c r="E134" s="4"/>
-    </row>
-    <row r="135" ht="13.55" customHeight="1">
-      <c r="A135" s="3"/>
-      <c r="B135" s="12"/>
-      <c r="C135" s="3"/>
-      <c r="D135" s="4"/>
-      <c r="E135" s="4"/>
-    </row>
-    <row r="136" ht="13.55" customHeight="1">
-      <c r="A136" s="7"/>
-      <c r="B136" s="7"/>
-      <c r="C136" s="7"/>
-      <c r="D136" s="4"/>
-      <c r="E136" s="4"/>
-    </row>
-    <row r="137" ht="16.6" customHeight="1">
-      <c r="A137" t="s" s="8">
-        <v>92</v>
-      </c>
-      <c r="B137" t="s" s="9">
-        <v>93</v>
-      </c>
-      <c r="C137" t="s" s="21">
-        <v>57</v>
-      </c>
-      <c r="D137" s="11"/>
-      <c r="E137" s="4"/>
-    </row>
-    <row r="138" ht="13.65" customHeight="1">
-      <c r="A138" s="12"/>
-      <c r="B138" t="s" s="13">
-        <v>94</v>
-      </c>
-      <c r="C138" s="12"/>
-      <c r="D138" s="4"/>
-      <c r="E138" s="4"/>
-    </row>
-    <row r="139" ht="13.55" customHeight="1">
-      <c r="A139" s="3"/>
-      <c r="B139" s="3"/>
-      <c r="C139" s="3"/>
-      <c r="D139" s="4"/>
-      <c r="E139" s="4"/>
-    </row>
-    <row r="140" ht="13.65" customHeight="1">
-      <c r="A140" s="3"/>
-      <c r="B140" t="s" s="14">
-        <v>95</v>
-      </c>
-      <c r="C140" s="3"/>
-      <c r="D140" s="4"/>
-      <c r="E140" s="4"/>
-    </row>
-    <row r="141" ht="13.65" customHeight="1">
-      <c r="A141" s="3"/>
-      <c r="B141" s="15"/>
-      <c r="C141" s="3"/>
-      <c r="D141" s="4"/>
-      <c r="E141" s="4"/>
-    </row>
-    <row r="142" ht="13.65" customHeight="1">
-      <c r="A142" s="3"/>
-      <c r="B142" t="s" s="14">
-        <v>96</v>
-      </c>
-      <c r="C142" s="3"/>
-      <c r="D142" s="4"/>
-      <c r="E142" s="4"/>
-    </row>
-    <row r="143" ht="13.55" customHeight="1">
-      <c r="A143" s="3"/>
-      <c r="B143" s="7"/>
-      <c r="C143" s="3"/>
-      <c r="D143" s="4"/>
-      <c r="E143" s="4"/>
-    </row>
-    <row r="144" ht="13.65" customHeight="1">
-      <c r="A144" s="16"/>
-      <c r="B144" t="s" s="17">
-        <v>13</v>
-      </c>
-      <c r="C144" s="18"/>
-      <c r="D144" s="4"/>
-      <c r="E144" s="4"/>
-    </row>
-    <row r="145" ht="13.55" customHeight="1">
-      <c r="A145" s="16"/>
-      <c r="B145" t="s" s="19">
-        <v>97</v>
-      </c>
-      <c r="C145" s="18"/>
-      <c r="D145" s="4"/>
-      <c r="E145" s="4"/>
-    </row>
-    <row r="146" ht="13.55" customHeight="1">
-      <c r="A146" s="16"/>
-      <c r="B146" t="s" s="19">
-        <v>98</v>
-      </c>
-      <c r="C146" s="18"/>
-      <c r="D146" s="4"/>
-      <c r="E146" s="4"/>
-    </row>
-    <row r="147" ht="13.55" customHeight="1">
-      <c r="A147" s="16"/>
-      <c r="B147" t="s" s="19">
-        <v>99</v>
-      </c>
-      <c r="C147" s="18"/>
-      <c r="D147" s="4"/>
-      <c r="E147" s="4"/>
-    </row>
-    <row r="148" ht="13.55" customHeight="1">
-      <c r="A148" s="3"/>
-      <c r="B148" s="12"/>
-      <c r="C148" s="3"/>
-      <c r="D148" s="4"/>
-      <c r="E148" s="4"/>
-    </row>
-    <row r="149" ht="13.55" customHeight="1">
-      <c r="A149" s="3"/>
-      <c r="B149" s="3"/>
-      <c r="C149" s="3"/>
-      <c r="D149" s="4"/>
-      <c r="E149" s="4"/>
-    </row>
-    <row r="150" ht="14.6" customHeight="1">
-      <c r="A150" t="s" s="22">
-        <v>100</v>
-      </c>
-      <c r="B150" s="3"/>
-      <c r="C150" s="3"/>
-      <c r="D150" s="4"/>
-      <c r="E150" s="4"/>
-    </row>
-    <row r="151" ht="13.55" customHeight="1">
-      <c r="A151" t="s" s="23">
-        <v>101</v>
-      </c>
-      <c r="B151" t="s" s="24">
-        <v>102</v>
-      </c>
-      <c r="C151" s="3"/>
-      <c r="D151" s="4"/>
-      <c r="E151" s="4"/>
-    </row>
-    <row r="152" ht="13.55" customHeight="1">
-      <c r="A152" t="s" s="23">
-        <v>103</v>
-      </c>
-      <c r="B152" t="s" s="24">
-        <v>104</v>
-      </c>
-      <c r="C152" s="3"/>
-      <c r="D152" s="4"/>
-      <c r="E152" s="4"/>
-    </row>
-    <row r="153" ht="13.55" customHeight="1">
-      <c r="A153" t="s" s="23">
-        <v>105</v>
-      </c>
-      <c r="B153" t="s" s="24">
-        <v>106</v>
-      </c>
-      <c r="C153" s="3"/>
-      <c r="D153" s="4"/>
-      <c r="E153" s="4"/>
-    </row>
-    <row r="154" ht="13.55" customHeight="1">
-      <c r="A154" t="s" s="23">
-        <v>107</v>
-      </c>
-      <c r="B154" t="s" s="24">
-        <v>108</v>
-      </c>
-      <c r="C154" s="3"/>
-      <c r="D154" s="4"/>
-      <c r="E154" s="4"/>
-    </row>
   </sheetData>
-  <mergeCells count="103">
+  <mergeCells count="79">
     <mergeCell ref="B91:C91"/>
     <mergeCell ref="B100:C100"/>
-    <mergeCell ref="B141:C141"/>
-    <mergeCell ref="B115:C115"/>
     <mergeCell ref="B93:C93"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B102:C102"/>
@@ -3056,66 +2644,50 @@
     <mergeCell ref="B77:C77"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B86:C86"/>
-    <mergeCell ref="B151:C151"/>
+    <mergeCell ref="B112:C112"/>
     <mergeCell ref="B61:C61"/>
     <mergeCell ref="B101:C101"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B78:C78"/>
-    <mergeCell ref="B112:C112"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B49:C49"/>
     <mergeCell ref="B64:C64"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B154:C154"/>
+    <mergeCell ref="B115:C115"/>
     <mergeCell ref="B35:C35"/>
     <mergeCell ref="B106:C106"/>
-    <mergeCell ref="B129:C129"/>
     <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B138:C138"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B140:C140"/>
-    <mergeCell ref="B130:C130"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B117:C117"/>
-    <mergeCell ref="B132:C132"/>
-    <mergeCell ref="B119:C119"/>
-    <mergeCell ref="B116:C116"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B103:C103"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B142:C142"/>
     <mergeCell ref="B89:C89"/>
     <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B144:C144"/>
-    <mergeCell ref="B153:C153"/>
+    <mergeCell ref="B114:C114"/>
     <mergeCell ref="B54:C54"/>
     <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B134:C134"/>
-    <mergeCell ref="B121:C121"/>
-    <mergeCell ref="B122:C122"/>
     <mergeCell ref="B56:C56"/>
     <mergeCell ref="B71:C71"/>
     <mergeCell ref="B105:C105"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="B43:C43"/>
     <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B120:C120"/>
     <mergeCell ref="B98:C98"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="B107:C107"/>
-    <mergeCell ref="A150:C150"/>
+    <mergeCell ref="A111:C111"/>
     <mergeCell ref="B57:C57"/>
     <mergeCell ref="B88:C88"/>
     <mergeCell ref="B44:C44"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B146:C146"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B108:C108"/>
     <mergeCell ref="B9:C9"/>
@@ -3124,28 +2696,22 @@
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B133:C133"/>
     <mergeCell ref="B45:C45"/>
     <mergeCell ref="B85:C85"/>
     <mergeCell ref="B94:C94"/>
-    <mergeCell ref="B126:C126"/>
     <mergeCell ref="B47:C47"/>
     <mergeCell ref="B62:C62"/>
     <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B152:C152"/>
+    <mergeCell ref="B113:C113"/>
     <mergeCell ref="B70:C70"/>
     <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B145:C145"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B73:C73"/>
     <mergeCell ref="B87:C87"/>
-    <mergeCell ref="B147:C147"/>
-    <mergeCell ref="B128:C128"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B74:C74"/>
     <mergeCell ref="B68:C68"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="B114:C114"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B50:C50"/>
   </mergeCells>

</xml_diff>